<commit_message>
BOM: volumen total por renglón y litros normales del gas
La columna de volumen mostraba el de una unidad (1 kg de N₂ = 800,5 L normales) al lado de cantidades de
gramos. Ahora es el volumen de la cantidad del renglón, igual que la masa total: 3,76 L normales de N₂ en el
ABC 1 kg y 0,045 L para 50 g de polvo. El gas lleva «(L normales)» en el nombre. El Word explica la columna.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/bom/FLAMA_BOM.xlsx
+++ b/salida/bom/FLAMA_BOM.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Volumen (L)</t>
+          <t>Volumen total (L)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -1399,7 +1399,7 @@
         <v>1.1</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="H27" s="18" t="n">
         <v>1</v>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D28" s="16" t="n">
@@ -1434,7 +1434,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>800.5</v>
+        <v>3.76235</v>
       </c>
       <c r="H28" s="18" t="n">
         <v>1</v>
@@ -2829,7 +2829,7 @@
         <v>1.1</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>2.318181818181818</v>
       </c>
       <c r="H72" s="18" t="n">
         <v>1</v>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D73" s="16" t="n">
@@ -2864,7 +2864,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G73" s="18" t="n">
-        <v>800.5</v>
+        <v>16.9706</v>
       </c>
       <c r="H73" s="18" t="n">
         <v>1</v>
@@ -4321,7 +4321,7 @@
         <v>1.1</v>
       </c>
       <c r="G119" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>4.681818181818182</v>
       </c>
       <c r="H119" s="18" t="n">
         <v>1</v>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D120" s="16" t="n">
@@ -4356,7 +4356,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G120" s="18" t="n">
-        <v>800.5</v>
+        <v>20.09255</v>
       </c>
       <c r="H120" s="18" t="n">
         <v>1</v>
@@ -5813,7 +5813,7 @@
         <v>1.1</v>
       </c>
       <c r="G166" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>9.227272727272727</v>
       </c>
       <c r="H166" s="18" t="n">
         <v>1</v>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="C167" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D167" s="16" t="n">
@@ -5848,7 +5848,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G167" s="18" t="n">
-        <v>800.5</v>
+        <v>47.0694</v>
       </c>
       <c r="H167" s="18" t="n">
         <v>1</v>
@@ -7445,7 +7445,7 @@
         <v>1.2</v>
       </c>
       <c r="G217" s="18" t="n">
-        <v>1.702083333333333</v>
+        <v>3.404166666666667</v>
       </c>
       <c r="H217" s="18" t="n">
         <v>2.0425</v>
@@ -7480,7 +7480,7 @@
         <v>7.85</v>
       </c>
       <c r="G218" s="18" t="n">
-        <v>0.2366114649681529</v>
+        <v>0.4732229299363057</v>
       </c>
       <c r="H218" s="18" t="n">
         <v>1.8574</v>
@@ -7719,7 +7719,7 @@
         <v>1.1</v>
       </c>
       <c r="G225" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>22.72727272727273</v>
       </c>
       <c r="H225" s="18" t="n">
         <v>1</v>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="C226" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D226" s="16" t="n">
@@ -7754,7 +7754,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G226" s="18" t="n">
-        <v>800.5</v>
+        <v>161.14065</v>
       </c>
       <c r="H226" s="18" t="n">
         <v>1</v>
@@ -9225,7 +9225,7 @@
         <v>1.2</v>
       </c>
       <c r="G272" s="18" t="n">
-        <v>2.780083333333334</v>
+        <v>5.560166666666667</v>
       </c>
       <c r="H272" s="18" t="n">
         <v>3.3361</v>
@@ -9260,7 +9260,7 @@
         <v>7.85</v>
       </c>
       <c r="G273" s="18" t="n">
-        <v>0.3320891719745223</v>
+        <v>0.6641783439490446</v>
       </c>
       <c r="H273" s="18" t="n">
         <v>2.6069</v>
@@ -9499,7 +9499,7 @@
         <v>1.1</v>
       </c>
       <c r="G280" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="H280" s="18" t="n">
         <v>1</v>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="C281" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D281" s="16" t="n">
@@ -9534,7 +9534,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G281" s="18" t="n">
-        <v>800.5</v>
+        <v>225.66095</v>
       </c>
       <c r="H281" s="18" t="n">
         <v>1</v>
@@ -11040,7 +11040,7 @@
         <v>1.2</v>
       </c>
       <c r="G328" s="18" t="n">
-        <v>2.780083333333334</v>
+        <v>5.560166666666667</v>
       </c>
       <c r="H328" s="18" t="n">
         <v>3.3361</v>
@@ -11075,7 +11075,7 @@
         <v>7.85</v>
       </c>
       <c r="G329" s="18" t="n">
-        <v>0.3320891719745223</v>
+        <v>0.6641783439490446</v>
       </c>
       <c r="H329" s="18" t="n">
         <v>2.6069</v>
@@ -11314,7 +11314,7 @@
         <v>1.1</v>
       </c>
       <c r="G336" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="H336" s="18" t="n">
         <v>1</v>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="C337" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D337" s="16" t="n">
@@ -11349,7 +11349,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G337" s="18" t="n">
-        <v>800.5</v>
+        <v>446.7590500000001</v>
       </c>
       <c r="H337" s="18" t="n">
         <v>1</v>
@@ -12855,7 +12855,7 @@
         <v>1.2</v>
       </c>
       <c r="G384" s="18" t="n">
-        <v>3.631166666666667</v>
+        <v>7.262333333333334</v>
       </c>
       <c r="H384" s="18" t="n">
         <v>4.3574</v>
@@ -12890,7 +12890,7 @@
         <v>7.85</v>
       </c>
       <c r="G385" s="18" t="n">
-        <v>0.3818980891719745</v>
+        <v>0.7637961783439491</v>
       </c>
       <c r="H385" s="18" t="n">
         <v>2.9979</v>
@@ -13129,7 +13129,7 @@
         <v>1.1</v>
       </c>
       <c r="G392" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>90.90909090909091</v>
       </c>
       <c r="H392" s="18" t="n">
         <v>1</v>
@@ -13149,7 +13149,7 @@
       </c>
       <c r="C393" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D393" s="16" t="n">
@@ -13164,7 +13164,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G393" s="18" t="n">
-        <v>800.5</v>
+        <v>415.37945</v>
       </c>
       <c r="H393" s="18" t="n">
         <v>1</v>
@@ -13642,7 +13642,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Volumen (L)</t>
+          <t>Volumen total (L)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -14608,7 +14608,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H30" s="18" t="n">
         <v>1</v>
@@ -14628,7 +14628,7 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D31" s="16" t="n">
@@ -14643,7 +14643,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>33.00268275862069</v>
       </c>
       <c r="H31" s="18" t="n">
         <v>1</v>
@@ -16104,7 +16104,7 @@
         <v>1</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H77" s="18" t="n">
         <v>1</v>
@@ -16139,7 +16139,7 @@
         <v>1.025</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H78" s="18" t="n">
         <v>1.025</v>
@@ -16159,7 +16159,7 @@
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D79" s="16" t="n">
@@ -16174,7 +16174,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>33.00268275862069</v>
       </c>
       <c r="H79" s="18" t="n">
         <v>1</v>
@@ -17705,7 +17705,7 @@
         <v>1.2</v>
       </c>
       <c r="G127" s="18" t="n">
-        <v>2.780083333333334</v>
+        <v>5.560166666666667</v>
       </c>
       <c r="H127" s="18" t="n">
         <v>3.3361</v>
@@ -17740,7 +17740,7 @@
         <v>7.85</v>
       </c>
       <c r="G128" s="18" t="n">
-        <v>0.3320891719745223</v>
+        <v>0.6641783439490446</v>
       </c>
       <c r="H128" s="18" t="n">
         <v>2.6069</v>
@@ -17979,7 +17979,7 @@
         <v>1</v>
       </c>
       <c r="G135" s="18" t="n">
-        <v>1</v>
+        <v>48.5</v>
       </c>
       <c r="H135" s="18" t="n">
         <v>1</v>
@@ -18014,7 +18014,7 @@
         <v>1.025</v>
       </c>
       <c r="G136" s="18" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H136" s="18" t="n">
         <v>1.025</v>
@@ -18034,7 +18034,7 @@
       </c>
       <c r="C137" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D137" s="16" t="n">
@@ -18049,7 +18049,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G137" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>97.77141379310345</v>
       </c>
       <c r="H137" s="18" t="n">
         <v>1</v>
@@ -19384,7 +19384,7 @@
         <v>0.9</v>
       </c>
       <c r="G179" s="18" t="n">
-        <v>1.111111111111111</v>
+        <v>5.722222222222223</v>
       </c>
       <c r="H179" s="18" t="n">
         <v>1</v>
@@ -19404,7 +19404,7 @@
       </c>
       <c r="C180" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D180" s="16" t="n">
@@ -19419,7 +19419,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G180" s="18" t="n">
-        <v>800.5</v>
+        <v>6.16385</v>
       </c>
       <c r="H180" s="18" t="n">
         <v>1</v>
@@ -20880,7 +20880,7 @@
         <v>1.3</v>
       </c>
       <c r="G226" s="18" t="n">
-        <v>1</v>
+        <v>6.09</v>
       </c>
       <c r="H226" s="18" t="n">
         <v>1.3</v>
@@ -20900,7 +20900,7 @@
       </c>
       <c r="C227" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D227" s="16" t="n">
@@ -20915,7 +20915,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G227" s="18" t="n">
-        <v>800.5</v>
+        <v>24.4953</v>
       </c>
       <c r="H227" s="18" t="n">
         <v>1</v>
@@ -22217,7 +22217,7 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="G268" s="18" t="n">
-        <v>1.48</v>
+        <v>2.96</v>
       </c>
       <c r="H268" s="18" t="n">
         <v>1</v>
@@ -23589,7 +23589,7 @@
         <v>0.6313131313131313</v>
       </c>
       <c r="G311" s="18" t="n">
-        <v>1.584</v>
+        <v>7.92</v>
       </c>
       <c r="H311" s="18" t="n">
         <v>1</v>
@@ -25015,7 +25015,7 @@
         <v>1.48</v>
       </c>
       <c r="G356" s="18" t="n">
-        <v>0.6756756756756757</v>
+        <v>3.378378378378378</v>
       </c>
       <c r="H356" s="18" t="n">
         <v>1</v>
@@ -25035,7 +25035,7 @@
       </c>
       <c r="C357" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Argón</t>
+          <t>Gas impulsor: Argón (L normales)</t>
         </is>
       </c>
       <c r="D357" s="16" t="n">
@@ -25050,7 +25050,7 @@
         <v>0.001784598911394664</v>
       </c>
       <c r="G357" s="18" t="n">
-        <v>560.35</v>
+        <v>21.74158</v>
       </c>
       <c r="H357" s="18" t="n">
         <v>1</v>
@@ -26511,7 +26511,7 @@
         <v>1</v>
       </c>
       <c r="G403" s="18" t="n">
-        <v>1</v>
+        <v>9.15</v>
       </c>
       <c r="H403" s="18" t="n">
         <v>1</v>
@@ -26531,7 +26531,7 @@
       </c>
       <c r="C404" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D404" s="16" t="n">
@@ -26546,7 +26546,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G404" s="18" t="n">
-        <v>800.5</v>
+        <v>48.3502</v>
       </c>
       <c r="H404" s="18" t="n">
         <v>1</v>
@@ -27115,7 +27115,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Volumen (L)</t>
+          <t>Volumen total (L)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -29275,7 +29275,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Volumen (L)</t>
+          <t>Volumen total (L)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -29425,7 +29425,7 @@
         <v>1.1</v>
       </c>
       <c r="G6" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="H6" s="18" t="n">
         <v>1</v>
@@ -29445,7 +29445,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D7" s="16" t="n">
@@ -29460,7 +29460,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>800.5</v>
+        <v>3.76235</v>
       </c>
       <c r="H7" s="18" t="n">
         <v>1</v>
@@ -29713,7 +29713,7 @@
         <v>1.1</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="H16" s="18" t="n">
         <v>1</v>
@@ -29733,7 +29733,7 @@
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D17" s="16" t="n">
@@ -29748,7 +29748,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>800.5</v>
+        <v>3.76235</v>
       </c>
       <c r="H17" s="18" t="n">
         <v>1</v>
@@ -30173,7 +30173,7 @@
         <v>1.1</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="H33" s="18" t="n">
         <v>1</v>
@@ -30193,7 +30193,7 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D34" s="16" t="n">
@@ -30208,7 +30208,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>800.5</v>
+        <v>16.9706</v>
       </c>
       <c r="H34" s="18" t="n">
         <v>1</v>
@@ -30461,7 +30461,7 @@
         <v>1.1</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>2.318181818181818</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>1</v>
@@ -30481,7 +30481,7 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D44" s="16" t="n">
@@ -30496,7 +30496,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>800.5</v>
+        <v>16.9706</v>
       </c>
       <c r="H44" s="18" t="n">
         <v>1</v>
@@ -30749,7 +30749,7 @@
         <v>1.1</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>2.272727272727272</v>
       </c>
       <c r="H53" s="18" t="n">
         <v>1</v>
@@ -30921,7 +30921,7 @@
         <v>1.1</v>
       </c>
       <c r="G60" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.1363636363636364</v>
       </c>
       <c r="H60" s="18" t="n">
         <v>1</v>
@@ -30941,7 +30941,7 @@
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D61" s="16" t="n">
@@ -30956,7 +30956,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>800.5</v>
+        <v>20.09255</v>
       </c>
       <c r="H61" s="18" t="n">
         <v>1</v>
@@ -31209,7 +31209,7 @@
         <v>1.1</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>4.681818181818182</v>
       </c>
       <c r="H70" s="18" t="n">
         <v>1</v>
@@ -31229,7 +31229,7 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D71" s="16" t="n">
@@ -31244,7 +31244,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>800.5</v>
+        <v>20.09255</v>
       </c>
       <c r="H71" s="18" t="n">
         <v>1</v>
@@ -31497,7 +31497,7 @@
         <v>1.1</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>4.545454545454545</v>
       </c>
       <c r="H80" s="18" t="n">
         <v>1</v>
@@ -31669,7 +31669,7 @@
         <v>1.1</v>
       </c>
       <c r="G87" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.1363636363636364</v>
       </c>
       <c r="H87" s="18" t="n">
         <v>1</v>
@@ -31689,7 +31689,7 @@
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
@@ -31704,7 +31704,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>800.5</v>
+        <v>47.0694</v>
       </c>
       <c r="H88" s="18" t="n">
         <v>1</v>
@@ -31957,7 +31957,7 @@
         <v>1.1</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>9.227272727272727</v>
       </c>
       <c r="H97" s="18" t="n">
         <v>1</v>
@@ -31977,7 +31977,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
@@ -31992,7 +31992,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>800.5</v>
+        <v>47.0694</v>
       </c>
       <c r="H98" s="18" t="n">
         <v>1</v>
@@ -32245,7 +32245,7 @@
         <v>1.1</v>
       </c>
       <c r="G107" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>9.09090909090909</v>
       </c>
       <c r="H107" s="18" t="n">
         <v>1</v>
@@ -32417,7 +32417,7 @@
         <v>1.1</v>
       </c>
       <c r="G114" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="H114" s="18" t="n">
         <v>1</v>
@@ -32437,7 +32437,7 @@
       </c>
       <c r="C115" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D115" s="16" t="n">
@@ -32452,7 +32452,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G115" s="18" t="n">
-        <v>800.5</v>
+        <v>161.14065</v>
       </c>
       <c r="H115" s="18" t="n">
         <v>1</v>
@@ -32705,7 +32705,7 @@
         <v>1.1</v>
       </c>
       <c r="G124" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>22.72727272727273</v>
       </c>
       <c r="H124" s="18" t="n">
         <v>1</v>
@@ -32725,7 +32725,7 @@
       </c>
       <c r="C125" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D125" s="16" t="n">
@@ -32740,7 +32740,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G125" s="18" t="n">
-        <v>800.5</v>
+        <v>161.14065</v>
       </c>
       <c r="H125" s="18" t="n">
         <v>1</v>
@@ -32993,7 +32993,7 @@
         <v>1.1</v>
       </c>
       <c r="G134" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>22.04545454545454</v>
       </c>
       <c r="H134" s="18" t="n">
         <v>1</v>
@@ -33165,7 +33165,7 @@
         <v>1.1</v>
       </c>
       <c r="G141" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>1.363636363636364</v>
       </c>
       <c r="H141" s="18" t="n">
         <v>1</v>
@@ -33185,7 +33185,7 @@
       </c>
       <c r="C142" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D142" s="16" t="n">
@@ -33200,7 +33200,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G142" s="18" t="n">
-        <v>800.5</v>
+        <v>225.66095</v>
       </c>
       <c r="H142" s="18" t="n">
         <v>1</v>
@@ -33453,7 +33453,7 @@
         <v>1.1</v>
       </c>
       <c r="G151" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="H151" s="18" t="n">
         <v>1</v>
@@ -33473,7 +33473,7 @@
       </c>
       <c r="C152" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D152" s="16" t="n">
@@ -33488,7 +33488,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G152" s="18" t="n">
-        <v>800.5</v>
+        <v>225.66095</v>
       </c>
       <c r="H152" s="18" t="n">
         <v>1</v>
@@ -33741,7 +33741,7 @@
         <v>1.1</v>
       </c>
       <c r="G161" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>44.09090909090909</v>
       </c>
       <c r="H161" s="18" t="n">
         <v>1</v>
@@ -33913,7 +33913,7 @@
         <v>1.1</v>
       </c>
       <c r="G168" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>1.909090909090909</v>
       </c>
       <c r="H168" s="18" t="n">
         <v>1</v>
@@ -33933,7 +33933,7 @@
       </c>
       <c r="C169" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D169" s="16" t="n">
@@ -33948,7 +33948,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G169" s="18" t="n">
-        <v>800.5</v>
+        <v>446.7590500000001</v>
       </c>
       <c r="H169" s="18" t="n">
         <v>1</v>
@@ -34201,7 +34201,7 @@
         <v>1.1</v>
       </c>
       <c r="G178" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="H178" s="18" t="n">
         <v>1</v>
@@ -34221,7 +34221,7 @@
       </c>
       <c r="C179" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D179" s="16" t="n">
@@ -34236,7 +34236,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G179" s="18" t="n">
-        <v>800.5</v>
+        <v>446.7590500000001</v>
       </c>
       <c r="H179" s="18" t="n">
         <v>1</v>
@@ -34489,7 +34489,7 @@
         <v>1.1</v>
       </c>
       <c r="G188" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>61.72727272727273</v>
       </c>
       <c r="H188" s="18" t="n">
         <v>1</v>
@@ -34661,7 +34661,7 @@
         <v>1.1</v>
       </c>
       <c r="G195" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>2.727272727272727</v>
       </c>
       <c r="H195" s="18" t="n">
         <v>1</v>
@@ -34681,7 +34681,7 @@
       </c>
       <c r="C196" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D196" s="16" t="n">
@@ -34696,7 +34696,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G196" s="18" t="n">
-        <v>800.5</v>
+        <v>415.37945</v>
       </c>
       <c r="H196" s="18" t="n">
         <v>1</v>
@@ -34949,7 +34949,7 @@
         <v>1.1</v>
       </c>
       <c r="G205" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>90.90909090909091</v>
       </c>
       <c r="H205" s="18" t="n">
         <v>1</v>
@@ -34969,7 +34969,7 @@
       </c>
       <c r="C206" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D206" s="16" t="n">
@@ -34984,7 +34984,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G206" s="18" t="n">
-        <v>800.5</v>
+        <v>415.37945</v>
       </c>
       <c r="H206" s="18" t="n">
         <v>1</v>
@@ -35237,7 +35237,7 @@
         <v>1.1</v>
       </c>
       <c r="G215" s="18" t="n">
-        <v>0.9090909090909091</v>
+        <v>88.18181818181817</v>
       </c>
       <c r="H215" s="18" t="n">
         <v>1</v>
@@ -35409,7 +35409,7 @@
         <v>1</v>
       </c>
       <c r="G222" s="18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H222" s="18" t="n">
         <v>1</v>
@@ -35429,7 +35429,7 @@
       </c>
       <c r="C223" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D223" s="16" t="n">
@@ -35444,7 +35444,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G223" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>33.00268275862069</v>
       </c>
       <c r="H223" s="18" t="n">
         <v>1</v>
@@ -35697,7 +35697,7 @@
         <v>1</v>
       </c>
       <c r="G232" s="18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H232" s="18" t="n">
         <v>1</v>
@@ -35717,7 +35717,7 @@
       </c>
       <c r="C233" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D233" s="16" t="n">
@@ -35732,7 +35732,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G233" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>33.00268275862069</v>
       </c>
       <c r="H233" s="18" t="n">
         <v>1</v>
@@ -36120,7 +36120,7 @@
         <v>1.025</v>
       </c>
       <c r="G248" s="18" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H248" s="18" t="n">
         <v>1.025</v>
@@ -36155,7 +36155,7 @@
         <v>1</v>
       </c>
       <c r="G249" s="18" t="n">
-        <v>1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H249" s="18" t="n">
         <v>1</v>
@@ -36175,7 +36175,7 @@
       </c>
       <c r="C250" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D250" s="16" t="n">
@@ -36190,7 +36190,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G250" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>33.00268275862069</v>
       </c>
       <c r="H250" s="18" t="n">
         <v>1</v>
@@ -36443,7 +36443,7 @@
         <v>1.025</v>
       </c>
       <c r="G259" s="18" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H259" s="18" t="n">
         <v>1.025</v>
@@ -36478,7 +36478,7 @@
         <v>1</v>
       </c>
       <c r="G260" s="18" t="n">
-        <v>1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H260" s="18" t="n">
         <v>1</v>
@@ -36498,7 +36498,7 @@
       </c>
       <c r="C261" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D261" s="16" t="n">
@@ -36513,7 +36513,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G261" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>33.00268275862069</v>
       </c>
       <c r="H261" s="18" t="n">
         <v>1</v>
@@ -36901,7 +36901,7 @@
         <v>1.025</v>
       </c>
       <c r="G276" s="18" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H276" s="18" t="n">
         <v>1.025</v>
@@ -36936,7 +36936,7 @@
         <v>1</v>
       </c>
       <c r="G277" s="18" t="n">
-        <v>1</v>
+        <v>48.5</v>
       </c>
       <c r="H277" s="18" t="n">
         <v>1</v>
@@ -36956,7 +36956,7 @@
       </c>
       <c r="C278" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D278" s="16" t="n">
@@ -36971,7 +36971,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G278" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>97.77141379310345</v>
       </c>
       <c r="H278" s="18" t="n">
         <v>1</v>
@@ -37224,7 +37224,7 @@
         <v>1.025</v>
       </c>
       <c r="G287" s="18" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H287" s="18" t="n">
         <v>1.025</v>
@@ -37259,7 +37259,7 @@
         <v>1</v>
       </c>
       <c r="G288" s="18" t="n">
-        <v>1</v>
+        <v>48.5</v>
       </c>
       <c r="H288" s="18" t="n">
         <v>1</v>
@@ -37279,7 +37279,7 @@
       </c>
       <c r="C289" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Aire comprimido</t>
+          <t>Gas impulsor: Aire comprimido (L normales)</t>
         </is>
       </c>
       <c r="D289" s="16" t="n">
@@ -37294,7 +37294,7 @@
         <v>0.001293834210761131</v>
       </c>
       <c r="G289" s="18" t="n">
-        <v>772.8965517241379</v>
+        <v>97.77141379310345</v>
       </c>
       <c r="H289" s="18" t="n">
         <v>1</v>
@@ -37682,7 +37682,7 @@
         <v>0.9</v>
       </c>
       <c r="G304" s="18" t="n">
-        <v>1.111111111111111</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H304" s="18" t="n">
         <v>1</v>
@@ -37702,7 +37702,7 @@
       </c>
       <c r="C305" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D305" s="16" t="n">
@@ -37717,7 +37717,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G305" s="18" t="n">
-        <v>800.5</v>
+        <v>6.16385</v>
       </c>
       <c r="H305" s="18" t="n">
         <v>1</v>
@@ -37970,7 +37970,7 @@
         <v>0.9</v>
       </c>
       <c r="G314" s="18" t="n">
-        <v>1.111111111111111</v>
+        <v>5.722222222222223</v>
       </c>
       <c r="H314" s="18" t="n">
         <v>1</v>
@@ -37990,7 +37990,7 @@
       </c>
       <c r="C315" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D315" s="16" t="n">
@@ -38005,7 +38005,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G315" s="18" t="n">
-        <v>800.5</v>
+        <v>6.16385</v>
       </c>
       <c r="H315" s="18" t="n">
         <v>1</v>
@@ -38258,7 +38258,7 @@
         <v>0.9</v>
       </c>
       <c r="G324" s="18" t="n">
-        <v>1.111111111111111</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="H324" s="18" t="n">
         <v>1</v>
@@ -38430,7 +38430,7 @@
         <v>1.3</v>
       </c>
       <c r="G331" s="18" t="n">
-        <v>1</v>
+        <v>6.09</v>
       </c>
       <c r="H331" s="18" t="n">
         <v>1.3</v>
@@ -38450,7 +38450,7 @@
       </c>
       <c r="C332" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D332" s="16" t="n">
@@ -38465,7 +38465,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G332" s="18" t="n">
-        <v>800.5</v>
+        <v>24.4953</v>
       </c>
       <c r="H332" s="18" t="n">
         <v>1</v>
@@ -38718,7 +38718,7 @@
         <v>1.3</v>
       </c>
       <c r="G341" s="18" t="n">
-        <v>1</v>
+        <v>6.09</v>
       </c>
       <c r="H341" s="18" t="n">
         <v>1.3</v>
@@ -38738,7 +38738,7 @@
       </c>
       <c r="C342" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D342" s="16" t="n">
@@ -38753,7 +38753,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G342" s="18" t="n">
-        <v>800.5</v>
+        <v>24.4953</v>
       </c>
       <c r="H342" s="18" t="n">
         <v>1</v>
@@ -39141,7 +39141,7 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="G357" s="18" t="n">
-        <v>1.48</v>
+        <v>0.148</v>
       </c>
       <c r="H357" s="18" t="n">
         <v>1</v>
@@ -39340,7 +39340,7 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="G364" s="18" t="n">
-        <v>1.48</v>
+        <v>2.96</v>
       </c>
       <c r="H364" s="18" t="n">
         <v>1</v>
@@ -39566,7 +39566,7 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="G372" s="18" t="n">
-        <v>1.48</v>
+        <v>2.96</v>
       </c>
       <c r="H372" s="18" t="n">
         <v>1</v>
@@ -39792,7 +39792,7 @@
         <v>0.6313131313131313</v>
       </c>
       <c r="G381" s="18" t="n">
-        <v>1.584</v>
+        <v>0.396</v>
       </c>
       <c r="H381" s="18" t="n">
         <v>1</v>
@@ -39991,7 +39991,7 @@
         <v>0.6313131313131313</v>
       </c>
       <c r="G388" s="18" t="n">
-        <v>1.584</v>
+        <v>7.92</v>
       </c>
       <c r="H388" s="18" t="n">
         <v>1</v>
@@ -40217,7 +40217,7 @@
         <v>0.6313131313131313</v>
       </c>
       <c r="G396" s="18" t="n">
-        <v>1.584</v>
+        <v>7.92</v>
       </c>
       <c r="H396" s="18" t="n">
         <v>1</v>
@@ -40443,7 +40443,7 @@
         <v>1.48</v>
       </c>
       <c r="G405" s="18" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.1013513513513513</v>
       </c>
       <c r="H405" s="18" t="n">
         <v>1</v>
@@ -40463,7 +40463,7 @@
       </c>
       <c r="C406" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Argón</t>
+          <t>Gas impulsor: Argón (L normales)</t>
         </is>
       </c>
       <c r="D406" s="16" t="n">
@@ -40478,7 +40478,7 @@
         <v>0.001784598911394664</v>
       </c>
       <c r="G406" s="18" t="n">
-        <v>560.35</v>
+        <v>21.74158</v>
       </c>
       <c r="H406" s="18" t="n">
         <v>1</v>
@@ -40731,7 +40731,7 @@
         <v>1.48</v>
       </c>
       <c r="G415" s="18" t="n">
-        <v>0.6756756756756757</v>
+        <v>3.378378378378378</v>
       </c>
       <c r="H415" s="18" t="n">
         <v>1</v>
@@ -40751,7 +40751,7 @@
       </c>
       <c r="C416" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: Argón</t>
+          <t>Gas impulsor: Argón (L normales)</t>
         </is>
       </c>
       <c r="D416" s="16" t="n">
@@ -40766,7 +40766,7 @@
         <v>0.001784598911394664</v>
       </c>
       <c r="G416" s="18" t="n">
-        <v>560.35</v>
+        <v>21.74158</v>
       </c>
       <c r="H416" s="18" t="n">
         <v>1</v>
@@ -41019,7 +41019,7 @@
         <v>1.48</v>
       </c>
       <c r="G425" s="18" t="n">
-        <v>0.6756756756756757</v>
+        <v>3.277027027027027</v>
       </c>
       <c r="H425" s="18" t="n">
         <v>1</v>
@@ -41191,7 +41191,7 @@
         <v>1</v>
       </c>
       <c r="G432" s="18" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="H432" s="18" t="n">
         <v>1</v>
@@ -41211,7 +41211,7 @@
       </c>
       <c r="C433" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D433" s="16" t="n">
@@ -41226,7 +41226,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G433" s="18" t="n">
-        <v>800.5</v>
+        <v>48.3502</v>
       </c>
       <c r="H433" s="18" t="n">
         <v>1</v>
@@ -41479,7 +41479,7 @@
         <v>1</v>
       </c>
       <c r="G442" s="18" t="n">
-        <v>1</v>
+        <v>9.15</v>
       </c>
       <c r="H442" s="18" t="n">
         <v>1</v>
@@ -41499,7 +41499,7 @@
       </c>
       <c r="C443" s="15" t="inlineStr">
         <is>
-          <t>Gas impulsor: N₂</t>
+          <t>Gas impulsor: N₂ (L normales)</t>
         </is>
       </c>
       <c r="D443" s="16" t="n">
@@ -41514,7 +41514,7 @@
         <v>0.001249219237976265</v>
       </c>
       <c r="G443" s="18" t="n">
-        <v>800.5</v>
+        <v>48.3502</v>
       </c>
       <c r="H443" s="18" t="n">
         <v>1</v>
@@ -41767,7 +41767,7 @@
         <v>1</v>
       </c>
       <c r="G452" s="18" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H452" s="18" t="n">
         <v>1</v>

</xml_diff>